<commit_message>
Replace unaccented 'aqui' across CLI prompts to prevent Windows terminal UTF-8 character corruption
</commit_message>
<xml_diff>
--- a/docs/peso y talla/Formato_Peso_Talla_LOS_CISNES_2026-08-13.xlsx
+++ b/docs/peso y talla/Formato_Peso_Talla_LOS_CISNES_2026-08-13.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="200">
   <si>
     <t xml:space="preserve">PROCESO 
 PROMOCIÓN Y PREVENCIÓN
@@ -168,69 +168,87 @@
     <t>10/07/2026</t>
   </si>
   <si>
-    <t>-0.26</t>
-  </si>
-  <si>
-    <t>NO</t>
+    <t>14.5</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>1018522203</t>
+  </si>
+  <si>
+    <t>LIAM MATHIAS</t>
+  </si>
+  <si>
+    <t>GOMEZ MUÑOZ</t>
+  </si>
+  <si>
+    <t>20/09/2023</t>
+  </si>
+  <si>
+    <t>02/02/2026</t>
+  </si>
+  <si>
+    <t>08/05/2026</t>
+  </si>
+  <si>
+    <t>12.7</t>
+  </si>
+  <si>
+    <t>89.9</t>
+  </si>
+  <si>
+    <t>18.1</t>
+  </si>
+  <si>
+    <t>1020849551</t>
+  </si>
+  <si>
+    <t>EMILY FERNANDA</t>
+  </si>
+  <si>
+    <t>CARDENAS NOGUERA</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>23/05/2021</t>
+  </si>
+  <si>
+    <t>15.3</t>
+  </si>
+  <si>
+    <t>99.6</t>
+  </si>
+  <si>
+    <t>17.1</t>
+  </si>
+  <si>
+    <t>1020849770</t>
+  </si>
+  <si>
+    <t>JHOAN MATEO</t>
+  </si>
+  <si>
+    <t>PINEDA VEGA</t>
+  </si>
+  <si>
+    <t>14/07/2021</t>
+  </si>
+  <si>
+    <t>15.7</t>
+  </si>
+  <si>
+    <t>97.6</t>
   </si>
   <si>
     <t>0</t>
   </si>
   <si>
-    <t>1018522203</t>
-  </si>
-  <si>
-    <t>LIAM MATHIAS</t>
-  </si>
-  <si>
-    <t>GOMEZ MUÑOZ</t>
-  </si>
-  <si>
-    <t>20/09/2023</t>
-  </si>
-  <si>
-    <t>02/02/2026</t>
-  </si>
-  <si>
-    <t>08/05/2026</t>
-  </si>
-  <si>
-    <t>-0.16</t>
-  </si>
-  <si>
-    <t>1020849551</t>
-  </si>
-  <si>
-    <t>EMILY FERNANDA</t>
-  </si>
-  <si>
-    <t>CARDENAS NOGUERA</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>23/05/2021</t>
-  </si>
-  <si>
-    <t>0.14</t>
-  </si>
-  <si>
-    <t>1020849770</t>
-  </si>
-  <si>
-    <t>JHOAN MATEO</t>
-  </si>
-  <si>
-    <t>PINEDA VEGA</t>
-  </si>
-  <si>
-    <t>14/07/2021</t>
-  </si>
-  <si>
-    <t>0.79</t>
-  </si>
-  <si>
     <t>1025332689</t>
   </si>
   <si>
@@ -243,7 +261,13 @@
     <t>06/11/2021</t>
   </si>
   <si>
-    <t>1.61</t>
+    <t>19.8</t>
+  </si>
+  <si>
+    <t>105.6</t>
+  </si>
+  <si>
+    <t>19.1</t>
   </si>
   <si>
     <t>1025332719</t>
@@ -258,7 +282,13 @@
     <t>13/12/2021</t>
   </si>
   <si>
-    <t>0.05</t>
+    <t>16.4</t>
+  </si>
+  <si>
+    <t>103.6</t>
+  </si>
+  <si>
+    <t>17</t>
   </si>
   <si>
     <t>1025332895</t>
@@ -273,6 +303,15 @@
     <t>18/03/2022</t>
   </si>
   <si>
+    <t>13.2</t>
+  </si>
+  <si>
+    <t>90.7</t>
+  </si>
+  <si>
+    <t>15.1</t>
+  </si>
+  <si>
     <t>1025333166</t>
   </si>
   <si>
@@ -285,7 +324,7 @@
     <t>11/08/2022</t>
   </si>
   <si>
-    <t>0.21</t>
+    <t>16.7</t>
   </si>
   <si>
     <t>1025333641</t>
@@ -300,7 +339,10 @@
     <t>01/05/2023</t>
   </si>
   <si>
-    <t>0.20</t>
+    <t>12.6</t>
+  </si>
+  <si>
+    <t>88.9</t>
   </si>
   <si>
     <t>1028410892</t>
@@ -315,7 +357,13 @@
     <t>13/12/2023</t>
   </si>
   <si>
-    <t>0.40</t>
+    <t>12.3</t>
+  </si>
+  <si>
+    <t>86.9</t>
+  </si>
+  <si>
+    <t>15</t>
   </si>
   <si>
     <t>1033125653</t>
@@ -330,7 +378,10 @@
     <t>21/09/2022</t>
   </si>
   <si>
-    <t>-0.12</t>
+    <t>13.6</t>
+  </si>
+  <si>
+    <t>93.6</t>
   </si>
   <si>
     <t>1033126594</t>
@@ -345,7 +396,13 @@
     <t>22/08/2024</t>
   </si>
   <si>
-    <t>0.69</t>
+    <t>12.1</t>
+  </si>
+  <si>
+    <t>84.7</t>
+  </si>
+  <si>
+    <t>16.3</t>
   </si>
   <si>
     <t>1249968406</t>
@@ -360,7 +417,13 @@
     <t>18/11/2022</t>
   </si>
   <si>
-    <t>-0.11</t>
+    <t>13.7</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>15.6</t>
   </si>
   <si>
     <t xml:space="preserve">Notas: </t>
@@ -2812,10 +2875,10 @@
         <v>56</v>
       </c>
       <c r="J17" s="43" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="K17" s="44" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="L17" s="44"/>
       <c r="M17" s="44"/>
@@ -2843,19 +2906,19 @@
         <v>3</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E18" s="41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F18" s="41" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G18" s="41" t="s">
         <v>54</v>
@@ -2864,13 +2927,13 @@
         <v>55</v>
       </c>
       <c r="I18" s="43" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J18" s="43" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="K18" s="44" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="L18" s="44"/>
       <c r="M18" s="44"/>
@@ -2898,19 +2961,19 @@
         <v>4</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E19" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G19" s="41" t="s">
         <v>54</v>
@@ -2919,13 +2982,13 @@
         <v>55</v>
       </c>
       <c r="I19" s="43" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J19" s="43" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="K19" s="44" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="L19" s="44"/>
       <c r="M19" s="44"/>
@@ -2953,19 +3016,19 @@
         <v>5</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C20" s="40" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D20" s="40" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E20" s="41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G20" s="41" t="s">
         <v>54</v>
@@ -2974,13 +3037,13 @@
         <v>55</v>
       </c>
       <c r="I20" s="43" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="J20" s="43" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="K20" s="44" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="L20" s="44"/>
       <c r="M20" s="44"/>
@@ -3008,19 +3071,19 @@
         <v>6</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D21" s="40" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G21" s="41" t="s">
         <v>54</v>
@@ -3029,13 +3092,13 @@
         <v>55</v>
       </c>
       <c r="I21" s="43" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="J21" s="43" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
       <c r="K21" s="44" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="L21" s="44"/>
       <c r="M21" s="44"/>
@@ -3063,19 +3126,19 @@
         <v>7</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E22" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G22" s="41" t="s">
         <v>54</v>
@@ -3084,13 +3147,13 @@
         <v>55</v>
       </c>
       <c r="I22" s="43" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="J22" s="43" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="K22" s="44" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="L22" s="44"/>
       <c r="M22" s="44"/>
@@ -3118,19 +3181,19 @@
         <v>8</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="D23" s="40" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="E23" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="G23" s="41" t="s">
         <v>54</v>
@@ -3139,13 +3202,13 @@
         <v>55</v>
       </c>
       <c r="I23" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="J23" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="J23" s="43" t="s">
-        <v>48</v>
-      </c>
       <c r="K23" s="44" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="L23" s="44"/>
       <c r="M23" s="44"/>
@@ -3173,19 +3236,19 @@
         <v>9</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E24" s="41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F24" s="41" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="G24" s="41" t="s">
         <v>54</v>
@@ -3194,13 +3257,13 @@
         <v>55</v>
       </c>
       <c r="I24" s="43" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="J24" s="43" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
       <c r="K24" s="44" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="L24" s="44"/>
       <c r="M24" s="44"/>
@@ -3228,19 +3291,19 @@
         <v>10</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="E25" s="41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F25" s="41" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="G25" s="41" t="s">
         <v>54</v>
@@ -3249,13 +3312,13 @@
         <v>55</v>
       </c>
       <c r="I25" s="43" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="J25" s="43" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
       <c r="K25" s="44" t="s">
-        <v>49</v>
+        <v>112</v>
       </c>
       <c r="L25" s="44"/>
       <c r="M25" s="44"/>
@@ -3283,19 +3346,19 @@
         <v>11</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="D26" s="40" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E26" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F26" s="41" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G26" s="41" t="s">
         <v>54</v>
@@ -3304,13 +3367,13 @@
         <v>55</v>
       </c>
       <c r="I26" s="43" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="J26" s="43" t="s">
-        <v>48</v>
+        <v>118</v>
       </c>
       <c r="K26" s="44" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="L26" s="44"/>
       <c r="M26" s="44"/>
@@ -3338,19 +3401,19 @@
         <v>12</v>
       </c>
       <c r="B27" s="40" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="D27" s="40" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="E27" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F27" s="41" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="G27" s="41" t="s">
         <v>54</v>
@@ -3359,13 +3422,13 @@
         <v>55</v>
       </c>
       <c r="I27" s="43" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="J27" s="43" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="K27" s="44" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="L27" s="44"/>
       <c r="M27" s="44"/>
@@ -3393,19 +3456,19 @@
         <v>13</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="E28" s="41" t="s">
         <v>43</v>
       </c>
       <c r="F28" s="41" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="G28" s="41" t="s">
         <v>54</v>
@@ -3414,13 +3477,13 @@
         <v>55</v>
       </c>
       <c r="I28" s="43" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="J28" s="43" t="s">
-        <v>48</v>
+        <v>131</v>
       </c>
       <c r="K28" s="44" t="s">
-        <v>49</v>
+        <v>132</v>
       </c>
       <c r="L28" s="44"/>
       <c r="M28" s="44"/>
@@ -3725,10 +3788,10 @@
     </row>
     <row r="37" ht="45.95" customHeight="1" spans="1:31" s="62" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="63" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B37" s="64" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="C37" s="65"/>
       <c r="D37" s="65"/>
@@ -3827,7 +3890,7 @@
     </row>
     <row r="40" ht="33.75" customHeight="1" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -3846,7 +3909,7 @@
       <c r="Q40" s="67"/>
       <c r="R40" s="67"/>
       <c r="S40" s="68" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="T40" s="68"/>
       <c r="U40" s="68"/>
@@ -3895,7 +3958,7 @@
     </row>
     <row r="42" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A42" s="71" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -3930,7 +3993,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A43" s="72" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="B43" s="72"/>
       <c r="C43" s="72"/>
@@ -3965,7 +4028,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A44" s="72" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="B44" s="72"/>
       <c r="C44" s="72"/>
@@ -4090,56 +4153,56 @@
       <c r="A4" s="75"/>
       <c r="B4" s="75"/>
       <c r="C4" s="76" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D4" s="76" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="75"/>
       <c r="B5" s="75"/>
       <c r="C5" s="78" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="D5" s="79"/>
     </row>
     <row r="6" ht="20.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="C6" s="81"/>
       <c r="D6" s="81"/>
     </row>
     <row r="7" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="80" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="B7" s="82" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="C7" s="82"/>
       <c r="D7" s="82"/>
     </row>
     <row r="8" ht="28.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B8" s="82" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C8" s="82"/>
       <c r="D8" s="82"/>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="80" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="B9" s="82" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="C9" s="82"/>
       <c r="D9" s="82"/>
@@ -4149,7 +4212,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="82" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="C10" s="82"/>
       <c r="D10" s="82"/>
@@ -4159,7 +4222,7 @@
         <v>17</v>
       </c>
       <c r="B11" s="82" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="C11" s="82"/>
       <c r="D11" s="82"/>
@@ -4169,7 +4232,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="82" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="C12" s="82"/>
       <c r="D12" s="82"/>
@@ -4179,7 +4242,7 @@
         <v>21</v>
       </c>
       <c r="B13" s="82" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="C13" s="82"/>
       <c r="D13" s="82"/>
@@ -4189,102 +4252,102 @@
         <v>22</v>
       </c>
       <c r="B14" s="82" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="C14" s="82"/>
       <c r="D14" s="82"/>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="80" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="B15" s="82" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="C15" s="82"/>
       <c r="D15" s="82"/>
     </row>
     <row r="16" ht="40.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="80" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="B16" s="82" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="C16" s="82"/>
       <c r="D16" s="82"/>
     </row>
     <row r="17" ht="50.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="80" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="B17" s="82" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="C17" s="82"/>
       <c r="D17" s="82"/>
     </row>
     <row r="18" ht="131.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="80" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B18" s="82" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C18" s="82"/>
       <c r="D18" s="82"/>
     </row>
     <row r="19" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="80" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="B19" s="82" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="C19" s="82"/>
       <c r="D19" s="82"/>
     </row>
     <row r="20" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="80" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="B20" s="82" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="C20" s="82"/>
       <c r="D20" s="82"/>
     </row>
     <row r="21" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="80" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="B21" s="82" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="C21" s="82"/>
       <c r="D21" s="82"/>
     </row>
     <row r="22" ht="95.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="80" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="B22" s="82" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="C22" s="82"/>
       <c r="D22" s="82"/>
     </row>
     <row r="23" ht="233.1" customHeight="1" spans="1:13" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="80" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="B23" s="82" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="C23" s="82"/>
       <c r="D23" s="82"/>
       <c r="E23" s="85" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="F23" s="85"/>
       <c r="G23" s="85"/>
@@ -4297,77 +4360,77 @@
     </row>
     <row r="24" ht="210.75" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="80" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
       <c r="B24" s="82" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="C24" s="82"/>
       <c r="D24" s="82"/>
     </row>
     <row r="25" ht="43.5" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="80" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="B25" s="82" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
       <c r="C25" s="82"/>
       <c r="D25" s="82"/>
     </row>
     <row r="26" ht="111.75" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="80" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="B26" s="82" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="C26" s="82"/>
       <c r="D26" s="82"/>
     </row>
     <row r="27" ht="63" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="80" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="B27" s="82" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="C27" s="82"/>
       <c r="D27" s="82"/>
     </row>
     <row r="28" ht="46.5" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="80" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="B28" s="82" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C28" s="82"/>
       <c r="D28" s="82"/>
     </row>
     <row r="29" ht="162" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="80" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="B29" s="82" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="C29" s="82"/>
       <c r="D29" s="82"/>
     </row>
     <row r="30" ht="105" customHeight="1" spans="1:4" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="80" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="B30" s="82" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="C30" s="82"/>
       <c r="D30" s="82"/>
     </row>
     <row r="31" ht="27" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="86" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="B31" s="86"/>
       <c r="C31" s="86"/>
@@ -4499,13 +4562,13 @@
         <v>1031859546</v>
       </c>
       <c r="M16" s="51" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="N16" s="51" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="O16" s="73" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="P16" s="73">
         <v>20.6</v>
@@ -4522,10 +4585,10 @@
         <v>1044510352</v>
       </c>
       <c r="M17" s="51" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="N17" s="51" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="O17" s="73" t="s">
         <v>43</v>
@@ -4545,10 +4608,10 @@
         <v>1031862104</v>
       </c>
       <c r="M18" s="51" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="N18" s="51" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="O18" s="73" t="s">
         <v>43</v>
@@ -4568,13 +4631,13 @@
         <v>1016972581</v>
       </c>
       <c r="M19" s="51" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="N19" s="51" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="O19" s="73" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="P19" s="73">
         <v>14.3</v>
@@ -4591,13 +4654,13 @@
         <v>1171713712</v>
       </c>
       <c r="M20" s="51" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="N20" s="51" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="O20" s="73" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="P20" s="73">
         <v>17.1</v>

</xml_diff>